<commit_message>
Updates to OMISSION workflow, adding BOLD
</commit_message>
<xml_diff>
--- a/inputs/CA Intertidal Barcode Data Received Updated 08062025.xlsx
+++ b/inputs/CA Intertidal Barcode Data Received Updated 08062025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mcallister/software/scripts/github/OMISSION/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD75C02A-1F9A-A142-B60D-A234DC2F29B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DC79E4E-D313-404F-8885-5717C08DE3B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7760" yWindow="-24900" windowWidth="40040" windowHeight="19580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="26780" yWindow="-28300" windowWidth="25540" windowHeight="23720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Recevied from Form" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="87">
   <si>
     <t>Project</t>
   </si>
@@ -291,6 +291,12 @@
   </si>
   <si>
     <t>Organized</t>
+  </si>
+  <si>
+    <t>IUCN_CA</t>
+  </si>
+  <si>
+    <t>CDFW_OPC</t>
   </si>
 </sst>
 </file>
@@ -641,7 +647,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AG925"/>
+  <dimension ref="A1:AG927"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" style="5" bestFit="1" customWidth="1"/>
@@ -1384,10 +1390,10 @@
       <c r="AF13" s="3"/>
       <c r="AG13" s="3"/>
     </row>
-    <row r="14" spans="1:33" ht="68">
+    <row r="14" spans="1:33" ht="16">
       <c r="A14" s="8"/>
-      <c r="B14" s="8" t="s">
-        <v>52</v>
+      <c r="B14" s="2" t="s">
+        <v>60</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>25</v>
@@ -1395,28 +1401,16 @@
       <c r="D14" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>12</v>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3" t="s">
+        <v>85</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="I14" s="8"/>
-      <c r="J14" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L14" s="9" t="s">
-        <v>54</v>
-      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
@@ -1439,10 +1433,10 @@
       <c r="AF14" s="3"/>
       <c r="AG14" s="3"/>
     </row>
-    <row r="15" spans="1:33" ht="68">
+    <row r="15" spans="1:33" ht="16">
       <c r="A15" s="8"/>
-      <c r="B15" s="8" t="s">
-        <v>52</v>
+      <c r="B15" s="2" t="s">
+        <v>60</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>25</v>
@@ -1450,28 +1444,16 @@
       <c r="D15" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>12</v>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3" t="s">
+        <v>86</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="I15" s="8"/>
-      <c r="J15" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L15" s="9" t="s">
-        <v>56</v>
-      </c>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
@@ -1494,7 +1476,7 @@
       <c r="AF15" s="3"/>
       <c r="AG15" s="3"/>
     </row>
-    <row r="16" spans="1:33" ht="17">
+    <row r="16" spans="1:33" ht="68">
       <c r="A16" s="8"/>
       <c r="B16" s="8" t="s">
         <v>52</v>
@@ -1512,10 +1494,10 @@
         <v>35</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I16" s="8"/>
       <c r="J16" s="3" t="s">
@@ -1525,7 +1507,7 @@
         <v>39</v>
       </c>
       <c r="L16" s="9" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
@@ -1549,19 +1531,39 @@
       <c r="AF16" s="3"/>
       <c r="AG16" s="3"/>
     </row>
-    <row r="17" spans="1:33" ht="16">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
+    <row r="17" spans="1:33" ht="68">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="I17" s="8"/>
+      <c r="J17" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>56</v>
+      </c>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
@@ -1584,19 +1586,39 @@
       <c r="AF17" s="3"/>
       <c r="AG17" s="3"/>
     </row>
-    <row r="18" spans="1:33" ht="14" customHeight="1">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
+    <row r="18" spans="1:33" ht="17">
+      <c r="A18" s="8"/>
+      <c r="B18" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="I18" s="8"/>
+      <c r="J18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L18" s="9" t="s">
+        <v>58</v>
+      </c>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
@@ -1654,7 +1676,7 @@
       <c r="AF19" s="3"/>
       <c r="AG19" s="3"/>
     </row>
-    <row r="20" spans="1:33" ht="16">
+    <row r="20" spans="1:33" ht="14" customHeight="1">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -33364,6 +33386,76 @@
       <c r="AF925" s="3"/>
       <c r="AG925" s="3"/>
     </row>
+    <row r="926" spans="1:33" ht="16">
+      <c r="A926" s="3"/>
+      <c r="B926" s="3"/>
+      <c r="C926" s="3"/>
+      <c r="D926" s="3"/>
+      <c r="E926" s="3"/>
+      <c r="F926" s="3"/>
+      <c r="G926" s="3"/>
+      <c r="H926" s="3"/>
+      <c r="I926" s="3"/>
+      <c r="J926" s="3"/>
+      <c r="K926" s="3"/>
+      <c r="L926" s="3"/>
+      <c r="M926" s="3"/>
+      <c r="N926" s="3"/>
+      <c r="O926" s="3"/>
+      <c r="P926" s="3"/>
+      <c r="Q926" s="3"/>
+      <c r="R926" s="3"/>
+      <c r="S926" s="3"/>
+      <c r="T926" s="3"/>
+      <c r="U926" s="3"/>
+      <c r="V926" s="3"/>
+      <c r="W926" s="3"/>
+      <c r="X926" s="3"/>
+      <c r="Y926" s="3"/>
+      <c r="Z926" s="3"/>
+      <c r="AA926" s="3"/>
+      <c r="AB926" s="3"/>
+      <c r="AC926" s="3"/>
+      <c r="AD926" s="3"/>
+      <c r="AE926" s="3"/>
+      <c r="AF926" s="3"/>
+      <c r="AG926" s="3"/>
+    </row>
+    <row r="927" spans="1:33" ht="16">
+      <c r="A927" s="3"/>
+      <c r="B927" s="3"/>
+      <c r="C927" s="3"/>
+      <c r="D927" s="3"/>
+      <c r="E927" s="3"/>
+      <c r="F927" s="3"/>
+      <c r="G927" s="3"/>
+      <c r="H927" s="3"/>
+      <c r="I927" s="3"/>
+      <c r="J927" s="3"/>
+      <c r="K927" s="3"/>
+      <c r="L927" s="3"/>
+      <c r="M927" s="3"/>
+      <c r="N927" s="3"/>
+      <c r="O927" s="3"/>
+      <c r="P927" s="3"/>
+      <c r="Q927" s="3"/>
+      <c r="R927" s="3"/>
+      <c r="S927" s="3"/>
+      <c r="T927" s="3"/>
+      <c r="U927" s="3"/>
+      <c r="V927" s="3"/>
+      <c r="W927" s="3"/>
+      <c r="X927" s="3"/>
+      <c r="Y927" s="3"/>
+      <c r="Z927" s="3"/>
+      <c r="AA927" s="3"/>
+      <c r="AB927" s="3"/>
+      <c r="AC927" s="3"/>
+      <c r="AD927" s="3"/>
+      <c r="AE927" s="3"/>
+      <c r="AF927" s="3"/>
+      <c r="AG927" s="3"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AG1" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AG16">
@@ -33373,9 +33465,9 @@
   <hyperlinks>
     <hyperlink ref="L11" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
     <hyperlink ref="K5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="L14" r:id="rId3" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="L15" r:id="rId4" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="L16" r:id="rId5" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="L16" r:id="rId3" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="L17" r:id="rId4" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="L18" r:id="rId5" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>